<commit_message>
docs: atualiza a planilha com o TDD final
</commit_message>
<xml_diff>
--- a/Tabela_US_BDD_TDD.xlsx
+++ b/Tabela_US_BDD_TDD.xlsx
@@ -517,7 +517,7 @@
 </t>
   </si>
   <si>
-    <t xml:space="preserve">        Usuario usuario = new Usuario("Ana");
+    <t xml:space="preserve">        Usuario usuario = new Usuario("Matheus", "matheus@email.com", "senha123");
         Curso curso = new Curso("Spring Boot Fundamentos");
         Matricula matricula = new Matricula(usuario, curso, false);</t>
   </si>
@@ -529,7 +529,7 @@
         assertEquals(3, usuario.getAssinatura().getCreditosCursos());</t>
   </si>
   <si>
-    <t xml:space="preserve">        Usuario usuario = new Usuario("Bruno");
+    <t xml:space="preserve">        Usuario usuario = new Usuario("Matheus", "matheus@email.com", "senha123");
         Curso curso = new Curso("Spring Boot Fundamentos");
         Matricula matricula = new Matricula(usuario, curso, false);</t>
   </si>
@@ -541,7 +541,7 @@
         assertEquals(0, usuario.getAssinatura().getCreditosCursos());</t>
   </si>
   <si>
-    <t xml:space="preserve">        Usuario usuario = new Usuario("Carla");
+    <t xml:space="preserve">        Usuario usuario = new Usuario("Rafael", "rafael@email.com", "senha123");
         Curso curso = new Curso("Java Basico");</t>
   </si>
   <si>
@@ -553,7 +553,7 @@
         assertEquals(0, usuario.getAssinatura().getCreditosCursos());</t>
   </si>
   <si>
-    <t xml:space="preserve">        Usuario usuario = new Usuario("Diego");
+    <t xml:space="preserve">        Usuario usuario = new Usuario("Rafael", "rafael@email.com", "senha123");
         Curso curso = new Curso("Java Basico");
         Matricula matricula = new Matricula(usuario, curso, false);</t>
   </si>
@@ -566,7 +566,7 @@
         assertEquals(0, usuario.getAssinatura().getCreditosCursos());</t>
   </si>
   <si>
-    <t xml:space="preserve">        Usuario usuario = new Usuario("Elisa");
+    <t xml:space="preserve">        Usuario usuario = new Usuario("Henrique", "henrique@email.com", "senha123");
         usuario.getAssinatura().adicionarCreditos(1);
         Curso curso = new Curso("Java Avancado");</t>
   </si>
@@ -579,7 +579,7 @@
         assertEquals(0, usuario.getAssinatura().getCreditosCursos());</t>
   </si>
   <si>
-    <t xml:space="preserve">        Usuario usuario = new Usuario("Fabio");
+    <t xml:space="preserve">        Usuario usuario = new Usuario("Henrique", "henrique@email.com", "senha123");
         Curso curso = new Curso("Java Avancado");</t>
   </si>
   <si>

</xml_diff>